<commit_message>
Cache total values in HS summary workbook
openpyxl writes formulas with no cached value, so the CELKEM row and the
control-total cells read back as empty in pandas, previewers and anything
else reading cached values. LibreOffice could not recalculate the file in
this environment (three runs, timing out at 300s and 900s on a 23-row
sheet), so the values are injected into the sheet XML directly.

The SUM formulas are left in place and still recalculate on open; each
cached value was computed from the four data rows and asserted against
the figures taken from the source documents (7 399 ks, 6 499,335 kg net,
7 474,535 kg gross, 764 cartons, 164 228,14 USD).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BgPoujjP8Cpe2ByV977Q1n
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Ponature_IV26-00126.xlsx
+++ b/output/HS_Code_Summary_Ponature_IV26-00126.xlsx
@@ -840,23 +840,23 @@
       <c r="D6" s="10" t="n"/>
       <c r="E6" s="11">
         <f>SUM(E2:E5)</f>
-        <v/>
+        <v>7399</v>
       </c>
       <c r="F6" s="12">
         <f>SUM(F2:F5)</f>
-        <v/>
+        <v>6499.335</v>
       </c>
       <c r="G6" s="12">
         <f>SUM(G2:G5)</f>
-        <v/>
+        <v>7474.535</v>
       </c>
       <c r="H6" s="11">
         <f>SUM(H2:H5)</f>
-        <v/>
+        <v>764</v>
       </c>
       <c r="I6" s="13">
         <f>SUM(I2:I5)</f>
-        <v/>
+        <v>164228.14</v>
       </c>
       <c r="J6" s="10" t="n"/>
       <c r="K6" s="8" t="n"/>
@@ -969,7 +969,7 @@
       </c>
       <c r="C19" s="18">
         <f>E6</f>
-        <v/>
+        <v>7399</v>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
       </c>
       <c r="C20" s="19">
         <f>I6</f>
-        <v/>
+        <v>164228.14</v>
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C21" s="20">
         <f>G6</f>
-        <v/>
+        <v>7474.535</v>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C22" s="18">
         <f>H6</f>
-        <v/>
+        <v>764</v>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>

</xml_diff>